<commit_message>
Agregar archivos de evaluación y teoría de física
</commit_message>
<xml_diff>
--- a/AUSENTE.xlsx
+++ b/AUSENTE.xlsx
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AppServ\www\rolux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46C5D859-403A-40B5-8CA0-EA6DF7F4FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11444025-EBB1-4470-8F0C-E4AD53874942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="2640" windowWidth="15375" windowHeight="8325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="15375" windowHeight="8325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Curso</t>
   </si>
@@ -60,61 +71,38 @@
     <t>I° A</t>
   </si>
   <si>
-    <t>Yuliana Mendicute</t>
-  </si>
-  <si>
-    <t>yuliana.mendicute@a.colsanjavier.cl</t>
-  </si>
-  <si>
-    <t>Mendicute Arechavala Juan Ignacio</t>
-  </si>
-  <si>
-    <t>jimendicute@eymgestorias.cl</t>
-  </si>
-  <si>
-    <t>Johnson Undurraga
-Maria Cecilia</t>
-  </si>
-  <si>
-    <t>cjohnson@colsanjavier.cl</t>
-  </si>
-  <si>
-    <t>a</t>
+    <t>ignacio.cano@a.colsanjavier.cl</t>
+  </si>
+  <si>
+    <t>Cano Mardones Claudio Leonel</t>
+  </si>
+  <si>
+    <t>claudiocano@sermar.cl</t>
+  </si>
+  <si>
+    <t>Nova Zenteno Cristina Lorena</t>
+  </si>
+  <si>
+    <t>cristy.nova@gmail.com</t>
+  </si>
+  <si>
+    <t>o</t>
+  </si>
+  <si>
+    <t>Ignacio Cano</t>
   </si>
   <si>
     <t>vradulovich@colsanjavier.cl</t>
   </si>
   <si>
     <t>Formación de imágenes en espejos planos, cóncavos y convexos mediante el trazado de rayos notables, la medición de distancias y el uso de la ecuación de Gauss para analizar las características de la imagen.</t>
-  </si>
-  <si>
-    <t>Juan Felipe Vergara Morales</t>
-  </si>
-  <si>
-    <t>juan.vergara@a.colsanjavier.cl</t>
-  </si>
-  <si>
-    <t>Vergara Bosman Felipe Edurado</t>
-  </si>
-  <si>
-    <t>vergarafelipe@gmail.com</t>
-  </si>
-  <si>
-    <t>Morales Vera
-Katty Daniela</t>
-  </si>
-  <si>
-    <t>kattymorales@gmail.com</t>
-  </si>
-  <si>
-    <t>o</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -129,24 +117,18 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -158,8 +140,14 @@
         <fgColor rgb="FF9CC2E5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor theme="0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -182,11 +170,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -197,17 +207,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -556,8 +568,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="43.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -591,67 +607,35 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" t="s">
         <v>18</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="J3" s="8" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar script para generar avisos de evaluaciones atrasadas y pruebas de importación cruzada en macOS
</commit_message>
<xml_diff>
--- a/AUSENTE.xlsx
+++ b/AUSENTE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11018"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AppServ\www\rolux\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MisApps/Documentos/www/rolux/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46C5D859-403A-40B5-8CA0-EA6DF7F4FB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC4DCA4-FEA4-464B-B076-5FBAAE56F6A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="2640" windowWidth="15375" windowHeight="8325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2640" yWindow="2640" windowWidth="25340" windowHeight="13240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -126,24 +126,29 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -214,74 +219,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -557,9 +494,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="22.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -591,7 +537,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -623,7 +569,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Agregar nueva clase de física sobre la Tierra y la Luna, incluir preguntas de autoevaluación y opciones múltiples en el documento de evaluación.
</commit_message>
<xml_diff>
--- a/AUSENTE.xlsx
+++ b/AUSENTE.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79E7ABF9-15F9-914B-9756-19C111F4E4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8F9495B-2638-4D21-86EF-C3DE70F25CB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="108">
   <si>
     <t>Enviar</t>
   </si>
@@ -69,9 +82,6 @@
   </si>
   <si>
     <t>a</t>
-  </si>
-  <si>
-    <t>Fri Sep 25 2026 21:00:00 GMT-0300 (hora de verano de Chile)</t>
   </si>
   <si>
     <t>Sat Dec 30 1899 03:47:15 GMT-0442 (hora de verano de Chile)</t>
@@ -97,9 +107,6 @@
     <t>heidiw2003@yahoo.com</t>
   </si>
   <si>
-    <t>Tue Sep 22 2026 21:00:00 GMT-0300 (hora de verano de Chile)</t>
-  </si>
-  <si>
     <t>Sat Dec 30 1899 10:47:15 GMT-0442 (hora de verano de Chile)</t>
   </si>
   <si>
@@ -245,6 +252,126 @@
   </si>
   <si>
     <t>patricia.sanhueza@colsanjavier.cl</t>
+  </si>
+  <si>
+    <t>Llanos Aicon Martina Andrea</t>
+  </si>
+  <si>
+    <t>Martínez Rivera Joaquín Salvador</t>
+  </si>
+  <si>
+    <t>Prado Núñez Isidora Amanda</t>
+  </si>
+  <si>
+    <t>Aravena Bucarey María Paz</t>
+  </si>
+  <si>
+    <t>Peña Linay Diego Alonso</t>
+  </si>
+  <si>
+    <t>Toro-Moreno Meriño Gonzalo Andrés</t>
+  </si>
+  <si>
+    <t>gonzalo.toro-moreno@a.colsanjavier.cl</t>
+  </si>
+  <si>
+    <t>Vásquez Sandoval Román Alonso</t>
+  </si>
+  <si>
+    <t>roman.vasquez@a.colsanjavier.cl</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>maria.aravena@a.colsanjavier.cl</t>
+    </r>
+  </si>
+  <si>
+    <t>hectoraravenar@gmail.com</t>
+  </si>
+  <si>
+    <t>sandrabucarey03@gmail.com</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>diego.pena@a.colsanjavier.cl</t>
+    </r>
+  </si>
+  <si>
+    <t>colibrispabotilleria@gmail.com</t>
+  </si>
+  <si>
+    <t>sergio_233@msn.com</t>
+  </si>
+  <si>
+    <t>mmerino270918@gmail.com</t>
+  </si>
+  <si>
+    <t>felipe.vasquez.vet@gmail.com</t>
+  </si>
+  <si>
+    <t>karin.sandoval.velasquez@gmail.com</t>
+  </si>
+  <si>
+    <t>I° C</t>
+  </si>
+  <si>
+    <t>Revillard San Martín Antonella Paz</t>
+  </si>
+  <si>
+    <t>antonella.revillard@a.colsanjavier.cl</t>
+  </si>
+  <si>
+    <t>Sayeg Muñoz Cristóbal Felipe</t>
+  </si>
+  <si>
+    <t>cristobal.sayeg@a.colsanjavier.cl</t>
+  </si>
+  <si>
+    <t>Chávez Vargas Sofía Isidora</t>
+  </si>
+  <si>
+    <t>sofia.chavez@a.colsanjavier.cl</t>
+  </si>
+  <si>
+    <t>III° A</t>
+  </si>
+  <si>
+    <t>III° C</t>
+  </si>
+  <si>
+    <t>martina.llanos@a.colsanjavier.cl</t>
+  </si>
+  <si>
+    <t>joaquin.martinez@a.colsanjavier.cl</t>
+  </si>
+  <si>
+    <t>isidora.prado@a.colsanjavier.cl</t>
+  </si>
+  <si>
+    <t>prado.riveros@gmail.com</t>
+  </si>
+  <si>
+    <t>paola.adriananunez73@gmail.com</t>
+  </si>
+  <si>
+    <t>mweisserv@gmail.com</t>
+  </si>
+  <si>
+    <t>carolina.rivera.t.cr@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -252,9 +379,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -284,8 +411,26 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1155CC"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -297,8 +442,14 @@
         <fgColor rgb="FF9CC2E5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor theme="0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -345,11 +496,74 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -385,23 +599,153 @@
     <xf numFmtId="14" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1119,6 +1463,84 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="85731" cy="179999"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3EFB48A4-FD4E-4F08-B618-E275148F421D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10153650" y="1152525"/>
+          <a:ext cx="85731" cy="179999"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="66680" cy="179999"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{49016681-043D-4E29-A157-B7B1B1BD3DBF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10153650" y="1152525"/>
+          <a:ext cx="66680" cy="179999"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1127,7 +1549,7 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr val="windowText" lastClr="171717"/>
       </a:dk1>
       <a:lt1>
         <a:sysClr val="window" lastClr="FFFFFF"/>
@@ -1444,19 +1866,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:V41"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5" style="13" customWidth="1"/>
-    <col min="2" max="2" width="13.5" customWidth="1"/>
-    <col min="3" max="3" width="42.1640625" customWidth="1"/>
-    <col min="4" max="7" width="13.5" customWidth="1"/>
-    <col min="8" max="8" width="13.5" style="18" customWidth="1"/>
-    <col min="9" max="9" width="16.1640625" style="18" customWidth="1"/>
-    <col min="10" max="22" width="13.5" customWidth="1"/>
+    <col min="1" max="1" width="13.42578125" style="13" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" customWidth="1"/>
+    <col min="3" max="3" width="42.140625" customWidth="1"/>
+    <col min="4" max="7" width="13.42578125" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" style="16" customWidth="1"/>
+    <col min="9" max="9" width="16.140625" style="16" customWidth="1"/>
+    <col min="10" max="22" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1502,7 +1924,7 @@
       <c r="U1" s="4"/>
       <c r="V1" s="4"/>
     </row>
-    <row r="2" spans="1:22" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>11</v>
       </c>
@@ -1524,14 +1946,14 @@
       <c r="G2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="18">
+        <v>46290</v>
+      </c>
+      <c r="I2" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="19" t="s">
+      <c r="J2" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>20</v>
       </c>
       <c r="K2" s="9">
         <v>-1</v>
@@ -1548,36 +1970,36 @@
       <c r="U2" s="4"/>
       <c r="V2" s="4"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D3" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>24</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>25</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" s="19" t="s">
-        <v>27</v>
+      <c r="H3" s="19">
+        <v>46287</v>
+      </c>
+      <c r="I3" s="20" t="s">
+        <v>25</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K3" s="9">
         <v>1</v>
@@ -1594,7 +2016,7 @@
       <c r="U3" s="4"/>
       <c r="V3" s="4"/>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>11</v>
       </c>
@@ -1602,28 +2024,28 @@
         <v>12</v>
       </c>
       <c r="C4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="F4" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="G4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" s="19" t="s">
-        <v>27</v>
+      <c r="H4" s="19">
+        <v>46287</v>
+      </c>
+      <c r="I4" s="20" t="s">
+        <v>25</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K4" s="9">
         <v>1</v>
@@ -1640,7 +2062,7 @@
       <c r="U4" s="4"/>
       <c r="V4" s="4"/>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>11</v>
       </c>
@@ -1648,26 +2070,26 @@
         <v>12</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E5" s="10"/>
       <c r="F5" s="10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="I5" s="19" t="s">
-        <v>27</v>
+      <c r="H5" s="19">
+        <v>46287</v>
+      </c>
+      <c r="I5" s="20" t="s">
+        <v>25</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K5" s="9">
         <v>1</v>
@@ -1684,7 +2106,7 @@
       <c r="U5" s="4"/>
       <c r="V5" s="4"/>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>11</v>
       </c>
@@ -1692,28 +2114,28 @@
         <v>12</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="F6" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>39</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" s="20" t="s">
-        <v>27</v>
+      <c r="H6" s="19">
+        <v>46287</v>
+      </c>
+      <c r="I6" s="21" t="s">
+        <v>25</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K6" s="9">
         <v>1</v>
@@ -1730,36 +2152,36 @@
       <c r="U6" s="4"/>
       <c r="V6" s="4"/>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="D7" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="E7" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="F7" s="11" t="s">
         <v>43</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>45</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="16" t="s">
+      <c r="H7" s="18">
+        <v>46290</v>
+      </c>
+      <c r="I7" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="20" t="s">
-        <v>19</v>
-      </c>
       <c r="J7" s="7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="K7" s="9">
         <v>0</v>
@@ -1776,36 +2198,36 @@
       <c r="U7" s="4"/>
       <c r="V7" s="4"/>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
-        <v>40</v>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="s">
+        <v>11</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C8" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E8" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="F8" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>50</v>
-      </c>
       <c r="G8" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H8" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" s="18">
+        <v>46290</v>
+      </c>
+      <c r="I8" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="20" t="s">
-        <v>19</v>
-      </c>
       <c r="J8" s="7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="K8" s="9">
         <v>0</v>
@@ -1822,36 +2244,36 @@
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A9" s="6" t="s">
-        <v>40</v>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A9" s="17" t="s">
+        <v>11</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C9" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="F9" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E9" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>54</v>
-      </c>
       <c r="G9" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H9" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="H9" s="18">
+        <v>46290</v>
+      </c>
+      <c r="I9" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="I9" s="20" t="s">
-        <v>19</v>
-      </c>
       <c r="J9" s="7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="K9" s="9">
         <v>0</v>
@@ -1868,36 +2290,36 @@
       <c r="U9" s="4"/>
       <c r="V9" s="4"/>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A10" s="6" t="s">
-        <v>40</v>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A10" s="17" t="s">
+        <v>11</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C10" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="F10" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="E10" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>58</v>
-      </c>
       <c r="G10" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H10" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="H10" s="18">
+        <v>46290</v>
+      </c>
+      <c r="I10" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="I10" s="20" t="s">
-        <v>19</v>
-      </c>
       <c r="J10" s="7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="K10" s="9">
         <v>0</v>
@@ -1914,36 +2336,36 @@
       <c r="U10" s="4"/>
       <c r="V10" s="4"/>
     </row>
-    <row r="11" spans="1:22" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
-        <v>40</v>
+    <row r="11" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="17" t="s">
+        <v>11</v>
       </c>
       <c r="B11" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="E11" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="F11" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="E11" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>63</v>
-      </c>
       <c r="G11" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H11" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="H11" s="18">
+        <v>46290</v>
+      </c>
+      <c r="I11" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="I11" s="20" t="s">
-        <v>19</v>
-      </c>
       <c r="J11" s="7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="K11" s="9">
         <v>0</v>
@@ -1960,36 +2382,36 @@
       <c r="U11" s="4"/>
       <c r="V11" s="4"/>
     </row>
-    <row r="12" spans="1:22" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12" s="6" t="s">
-        <v>40</v>
+    <row r="12" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="17" t="s">
+        <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="F12" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="E12" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>67</v>
-      </c>
       <c r="G12" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H12" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="H12" s="18">
+        <v>46290</v>
+      </c>
+      <c r="I12" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="I12" s="20" t="s">
-        <v>19</v>
-      </c>
       <c r="J12" s="7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="K12" s="9">
         <v>0</v>
@@ -2006,36 +2428,36 @@
       <c r="U12" s="4"/>
       <c r="V12" s="4"/>
     </row>
-    <row r="13" spans="1:22" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="6" t="s">
-        <v>40</v>
+    <row r="13" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="17" t="s">
+        <v>11</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C13" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="E13" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="F13" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="E13" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>71</v>
-      </c>
       <c r="G13" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H13" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="H13" s="18">
+        <v>46290</v>
+      </c>
+      <c r="I13" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="20" t="s">
-        <v>19</v>
-      </c>
       <c r="J13" s="7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="K13" s="9">
         <v>0</v>
@@ -2052,36 +2474,36 @@
       <c r="U13" s="4"/>
       <c r="V13" s="4"/>
     </row>
-    <row r="14" spans="1:22" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C14" s="7" t="s">
+    <row r="14" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="C14" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="D14" s="51" t="s">
+        <v>71</v>
+      </c>
+      <c r="E14" s="38" t="s">
         <v>72</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="F14" s="38" t="s">
         <v>73</v>
       </c>
-      <c r="E14" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="G14" s="5" t="s">
+      <c r="G14" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="16" t="s">
+      <c r="H14" s="18">
+        <v>46290</v>
+      </c>
+      <c r="I14" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="I14" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="J14" s="7" t="s">
-        <v>46</v>
+      <c r="J14" s="25" t="s">
+        <v>44</v>
       </c>
       <c r="K14" s="9">
         <v>0</v>
@@ -2098,17 +2520,27 @@
       <c r="U14" s="4"/>
       <c r="V14" s="4"/>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A15" s="12"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="17"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="4"/>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A15" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" s="30" t="s">
+        <v>101</v>
+      </c>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" s="31"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="30"/>
       <c r="K15" s="4"/>
       <c r="L15" s="4"/>
       <c r="M15" s="4"/>
@@ -2122,17 +2554,31 @@
       <c r="U15" s="4"/>
       <c r="V15" s="4"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A16" s="12"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="4"/>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A16" s="39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="47" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="41" t="s">
+        <v>102</v>
+      </c>
+      <c r="E16" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="F16" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="G16" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="H16" s="31"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="30"/>
       <c r="K16" s="4"/>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
@@ -2146,17 +2592,31 @@
       <c r="U16" s="4"/>
       <c r="V16" s="4"/>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A17" s="12"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="4"/>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A17" s="39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="47" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="E17" s="41" t="s">
+        <v>104</v>
+      </c>
+      <c r="F17" s="41" t="s">
+        <v>105</v>
+      </c>
+      <c r="G17" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="31"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="30"/>
       <c r="K17" s="4"/>
       <c r="L17" s="4"/>
       <c r="M17" s="4"/>
@@ -2170,17 +2630,31 @@
       <c r="U17" s="4"/>
       <c r="V17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A18" s="12"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="4"/>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A18" s="39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="C18" s="48" t="s">
+        <v>77</v>
+      </c>
+      <c r="D18" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" s="40" t="s">
+        <v>84</v>
+      </c>
+      <c r="F18" s="40" t="s">
+        <v>85</v>
+      </c>
+      <c r="G18" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="31"/>
+      <c r="I18" s="32"/>
+      <c r="J18" s="30"/>
       <c r="K18" s="4"/>
       <c r="L18" s="4"/>
       <c r="M18" s="4"/>
@@ -2194,17 +2668,31 @@
       <c r="U18" s="4"/>
       <c r="V18" s="4"/>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A19" s="12"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="17"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="4"/>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A19" s="39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="C19" s="48" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" s="41" t="s">
+        <v>86</v>
+      </c>
+      <c r="E19" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="F19" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="G19" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="H19" s="31"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="30"/>
       <c r="K19" s="4"/>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -2218,17 +2706,31 @@
       <c r="U19" s="4"/>
       <c r="V19" s="4"/>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A20" s="12"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="4"/>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A20" s="39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="C20" s="48" t="s">
+        <v>79</v>
+      </c>
+      <c r="D20" s="41" t="s">
+        <v>80</v>
+      </c>
+      <c r="E20" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="F20" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="G20" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="H20" s="31"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="30"/>
       <c r="K20" s="4"/>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -2242,17 +2744,31 @@
       <c r="U20" s="4"/>
       <c r="V20" s="4"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A21" s="12"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="17"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="4"/>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A21" s="39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="C21" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" s="42" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="40" t="s">
+        <v>91</v>
+      </c>
+      <c r="G21" s="43" t="s">
+        <v>30</v>
+      </c>
+      <c r="H21" s="31"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="30"/>
       <c r="K21" s="4"/>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -2266,18 +2782,40 @@
       <c r="U21" s="4"/>
       <c r="V21" s="4"/>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A22" s="12"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A22" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22" s="34" t="s">
+        <v>41</v>
+      </c>
+      <c r="E22" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="F22" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="G22" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" s="36">
+        <v>46295</v>
+      </c>
+      <c r="I22" s="37">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="J22" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="K22" s="9">
+        <v>0</v>
+      </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
       <c r="N22" s="4"/>
@@ -2290,17 +2828,25 @@
       <c r="U22" s="4"/>
       <c r="V22" s="4"/>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A23" s="12"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="4"/>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A23" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="C23" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="D23" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="E23" s="30"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="44"/>
+      <c r="I23" s="44"/>
+      <c r="J23" s="30"/>
       <c r="K23" s="4"/>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -2314,17 +2860,25 @@
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A24" s="12"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="17"/>
-      <c r="I24" s="17"/>
-      <c r="J24" s="4"/>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A24" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="C24" s="30" t="s">
+        <v>95</v>
+      </c>
+      <c r="D24" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="44"/>
+      <c r="I24" s="44"/>
+      <c r="J24" s="30"/>
       <c r="K24" s="4"/>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -2338,17 +2892,25 @@
       <c r="U24" s="4"/>
       <c r="V24" s="4"/>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A25" s="12"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="4"/>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A25" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" s="29" t="s">
+        <v>100</v>
+      </c>
+      <c r="C25" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="D25" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="E25" s="30"/>
+      <c r="F25" s="30"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="44"/>
+      <c r="I25" s="44"/>
+      <c r="J25" s="30"/>
       <c r="K25" s="4"/>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -2362,7 +2924,7 @@
       <c r="U25" s="4"/>
       <c r="V25" s="4"/>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" s="12"/>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -2370,8 +2932,8 @@
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
+      <c r="H26" s="15"/>
+      <c r="I26" s="15"/>
       <c r="J26" s="4"/>
       <c r="K26" s="4"/>
       <c r="L26" s="4"/>
@@ -2386,7 +2948,7 @@
       <c r="U26" s="4"/>
       <c r="V26" s="4"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" s="12"/>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
@@ -2394,8 +2956,8 @@
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
-      <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
+      <c r="H27" s="15"/>
+      <c r="I27" s="15"/>
       <c r="J27" s="4"/>
       <c r="K27" s="4"/>
       <c r="L27" s="4"/>
@@ -2410,7 +2972,7 @@
       <c r="U27" s="4"/>
       <c r="V27" s="4"/>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28" s="12"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -2418,8 +2980,8 @@
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
-      <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
+      <c r="H28" s="15"/>
+      <c r="I28" s="15"/>
       <c r="J28" s="4"/>
       <c r="K28" s="4"/>
       <c r="L28" s="4"/>
@@ -2434,7 +2996,7 @@
       <c r="U28" s="4"/>
       <c r="V28" s="4"/>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A29" s="12"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
@@ -2442,8 +3004,8 @@
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
-      <c r="H29" s="17"/>
-      <c r="I29" s="17"/>
+      <c r="H29" s="15"/>
+      <c r="I29" s="15"/>
       <c r="J29" s="4"/>
       <c r="K29" s="4"/>
       <c r="L29" s="4"/>
@@ -2458,7 +3020,7 @@
       <c r="U29" s="4"/>
       <c r="V29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" s="12"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -2466,8 +3028,8 @@
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
-      <c r="H30" s="17"/>
-      <c r="I30" s="17"/>
+      <c r="H30" s="15"/>
+      <c r="I30" s="15"/>
       <c r="J30" s="4"/>
       <c r="K30" s="4"/>
       <c r="L30" s="4"/>
@@ -2482,7 +3044,7 @@
       <c r="U30" s="4"/>
       <c r="V30" s="4"/>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31" s="12"/>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -2490,8 +3052,8 @@
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
-      <c r="H31" s="17"/>
-      <c r="I31" s="17"/>
+      <c r="H31" s="15"/>
+      <c r="I31" s="15"/>
       <c r="J31" s="4"/>
       <c r="K31" s="4"/>
       <c r="L31" s="4"/>
@@ -2506,7 +3068,7 @@
       <c r="U31" s="4"/>
       <c r="V31" s="4"/>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" s="12"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
@@ -2514,8 +3076,8 @@
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
-      <c r="H32" s="17"/>
-      <c r="I32" s="17"/>
+      <c r="H32" s="15"/>
+      <c r="I32" s="15"/>
       <c r="J32" s="4"/>
       <c r="K32" s="4"/>
       <c r="L32" s="4"/>
@@ -2530,7 +3092,7 @@
       <c r="U32" s="4"/>
       <c r="V32" s="4"/>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" s="12"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
@@ -2538,8 +3100,8 @@
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
-      <c r="H33" s="17"/>
-      <c r="I33" s="17"/>
+      <c r="H33" s="15"/>
+      <c r="I33" s="15"/>
       <c r="J33" s="4"/>
       <c r="K33" s="4"/>
       <c r="L33" s="4"/>
@@ -2554,7 +3116,7 @@
       <c r="U33" s="4"/>
       <c r="V33" s="4"/>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34" s="12"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -2562,8 +3124,8 @@
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
-      <c r="H34" s="17"/>
-      <c r="I34" s="17"/>
+      <c r="H34" s="15"/>
+      <c r="I34" s="15"/>
       <c r="J34" s="4"/>
       <c r="K34" s="4"/>
       <c r="L34" s="4"/>
@@ -2578,7 +3140,7 @@
       <c r="U34" s="4"/>
       <c r="V34" s="4"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A35" s="12"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -2586,8 +3148,8 @@
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
-      <c r="H35" s="17"/>
-      <c r="I35" s="17"/>
+      <c r="H35" s="15"/>
+      <c r="I35" s="15"/>
       <c r="J35" s="4"/>
       <c r="K35" s="4"/>
       <c r="L35" s="4"/>
@@ -2602,7 +3164,7 @@
       <c r="U35" s="4"/>
       <c r="V35" s="4"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -2610,8 +3172,8 @@
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
-      <c r="H36" s="17"/>
-      <c r="I36" s="17"/>
+      <c r="H36" s="15"/>
+      <c r="I36" s="15"/>
       <c r="J36" s="4"/>
       <c r="K36" s="4"/>
       <c r="L36" s="4"/>
@@ -2626,7 +3188,7 @@
       <c r="U36" s="4"/>
       <c r="V36" s="4"/>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" s="12"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -2634,8 +3196,8 @@
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
       <c r="G37" s="4"/>
-      <c r="H37" s="17"/>
-      <c r="I37" s="17"/>
+      <c r="H37" s="15"/>
+      <c r="I37" s="15"/>
       <c r="J37" s="4"/>
       <c r="K37" s="4"/>
       <c r="L37" s="4"/>
@@ -2650,7 +3212,7 @@
       <c r="U37" s="4"/>
       <c r="V37" s="4"/>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" s="12"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -2658,8 +3220,8 @@
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
-      <c r="H38" s="17"/>
-      <c r="I38" s="17"/>
+      <c r="H38" s="15"/>
+      <c r="I38" s="15"/>
       <c r="J38" s="4"/>
       <c r="K38" s="4"/>
       <c r="L38" s="4"/>
@@ -2674,7 +3236,7 @@
       <c r="U38" s="4"/>
       <c r="V38" s="4"/>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A39" s="12"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -2682,8 +3244,8 @@
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
-      <c r="H39" s="17"/>
-      <c r="I39" s="17"/>
+      <c r="H39" s="15"/>
+      <c r="I39" s="15"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
       <c r="L39" s="4"/>
@@ -2698,7 +3260,7 @@
       <c r="U39" s="4"/>
       <c r="V39" s="4"/>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A40" s="12"/>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
@@ -2706,8 +3268,8 @@
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
-      <c r="H40" s="17"/>
-      <c r="I40" s="17"/>
+      <c r="H40" s="15"/>
+      <c r="I40" s="15"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
       <c r="L40" s="4"/>
@@ -2722,6 +3284,30 @@
       <c r="U40" s="4"/>
       <c r="V40" s="4"/>
     </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A41" s="12"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="15"/>
+      <c r="I41" s="15"/>
+      <c r="J41" s="4"/>
+      <c r="K41" s="4"/>
+      <c r="L41" s="4"/>
+      <c r="M41" s="4"/>
+      <c r="N41" s="4"/>
+      <c r="O41" s="4"/>
+      <c r="P41" s="4"/>
+      <c r="Q41" s="4"/>
+      <c r="R41" s="4"/>
+      <c r="S41" s="4"/>
+      <c r="T41" s="4"/>
+      <c r="U41" s="4"/>
+      <c r="V41" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>